<commit_message>
Show the Utair quote status and offered price on the HBS list.
Keep every original column unchanged and fill only the two new columns from quotes sent since 5 August 2026.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/HBS_List_оборот_с_предложениями.xlsx
+++ b/HBS_List_оборот_с_предложениями.xlsx
@@ -472,7 +472,7 @@
     <col width="11.53125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="7.6640625" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="26.1328125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -539,7 +539,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -647,7 +647,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>NE, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G27" s="3" t="n">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G29" s="3" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G32" s="3" t="n">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SV, RE</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>OH, SV, RP, INSP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>INSP/TEST</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G42" s="3" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SV, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G50" s="3" t="n">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G51" s="3" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G58" s="3" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>SV, RE</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>OH, RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G94" s="3" t="n">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G96" s="3" t="n">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>OH, RP, TEST</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G113" s="3" t="n">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>OH, SV, RP, TEST</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G158" s="3" t="n">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G164" s="3" t="n">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G168" s="3" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>NE, OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G194" s="3" t="n">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G195" s="3" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G203" s="3" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -6318,7 +6318,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G215" s="3" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G218" s="3" t="n">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G219" s="3" t="n">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>SV, INSP</t>
+          <t>5. Есть интерес; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G233" s="3" t="n">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>NE, OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G253" s="3" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>SV, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G265" s="3" t="n">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G270" s="3" t="n">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G273" s="3" t="n">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G281" s="3" t="n">
@@ -8825,7 +8825,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G310" s="3" t="n">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G319" s="3" t="n">
@@ -9091,7 +9091,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G320" s="3" t="n">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G325" s="3" t="n">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -9727,7 +9727,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G344" s="3" t="n">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G367" s="3" t="n">
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>SV, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G379" s="3" t="n">
@@ -10686,7 +10686,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>NE, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G401" s="3" t="n">
@@ -11459,7 +11459,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G410" s="3" t="n">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G416" s="3" t="n">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>NE, OH, SV, RP, INSP, INSP/TEST</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G425" s="3" t="n">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G426" s="3" t="n">
@@ -12206,7 +12206,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G437" s="3" t="n">
@@ -12389,7 +12389,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G444" s="3" t="n">
@@ -12647,7 +12647,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G454" s="3" t="n">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>NE, OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="F485" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G485" s="3" t="n">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G486" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G488" s="3" t="n">
@@ -14401,7 +14401,7 @@
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>SV, RP, INSP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G522" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G548" s="3" t="n">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G551" t="inlineStr">
@@ -15679,7 +15679,7 @@
       </c>
       <c r="F572" t="inlineStr">
         <is>
-          <t>SV, RP</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G572" t="inlineStr">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>OH, SV, INSP, TEST</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G597" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G603" s="3" t="n">
@@ -16557,7 +16557,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>SV, RP</t>
+          <t>5. Есть интерес</t>
         </is>
       </c>
       <c r="G606" s="3" t="n">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G614" s="3" t="n">
@@ -17423,7 +17423,7 @@
       </c>
       <c r="F640" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G640" s="3" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="F657" t="inlineStr">
         <is>
-          <t>NE, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G657" t="inlineStr">
@@ -17966,7 +17966,7 @@
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G661" s="3" t="n">
@@ -18124,7 +18124,7 @@
       </c>
       <c r="F667" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G667" s="3" t="n">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G672" t="inlineStr">
@@ -18542,7 +18542,7 @@
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G683" s="3" t="n">
@@ -18625,7 +18625,7 @@
       </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G686" t="inlineStr">
@@ -19285,7 +19285,7 @@
       </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>OH, SV, RP</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G712" t="inlineStr">
@@ -19445,7 +19445,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G718" s="3" t="n">
@@ -19528,7 +19528,7 @@
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G721" s="3" t="n">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="F722" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G722" s="3" t="n">
@@ -19819,7 +19819,7 @@
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G732" t="inlineStr">
@@ -20004,7 +20004,7 @@
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G739" s="3" t="n">
@@ -20212,7 +20212,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>OH, RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G747" t="inlineStr">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="F750" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G750" s="3" t="n">
@@ -20580,7 +20580,7 @@
       </c>
       <c r="F761" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G761" s="3" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G768" s="3" t="n">
@@ -20821,7 +20821,7 @@
       </c>
       <c r="F770" t="inlineStr">
         <is>
-          <t>OH, RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G770" t="inlineStr">
@@ -21106,7 +21106,7 @@
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>OH, SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G781" t="inlineStr">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="F797" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G797" s="3" t="n">
@@ -22249,7 +22249,7 @@
       </c>
       <c r="F826" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G826" s="3" t="n">
@@ -22382,7 +22382,7 @@
       </c>
       <c r="F831" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G831" t="inlineStr">
@@ -22417,7 +22417,7 @@
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G832" t="inlineStr">
@@ -22852,7 +22852,7 @@
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G849" s="3" t="n">
@@ -22960,7 +22960,7 @@
       </c>
       <c r="F853" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G853" s="3" t="n">
@@ -23018,7 +23018,7 @@
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G855" s="3" t="n">
@@ -23051,7 +23051,7 @@
       </c>
       <c r="F856" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G856" s="3" t="n">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>OH, SV, TEST</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G859" t="inlineStr">
@@ -24619,7 +24619,7 @@
       </c>
       <c r="F918" t="inlineStr">
         <is>
-          <t>RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G918" s="3" t="n">
@@ -24952,7 +24952,7 @@
       </c>
       <c r="F931" t="inlineStr">
         <is>
-          <t>SV</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G931" s="3" t="n">
@@ -25110,7 +25110,7 @@
       </c>
       <c r="F937" t="inlineStr">
         <is>
-          <t>FN, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G937" t="inlineStr">
@@ -25145,7 +25145,7 @@
       </c>
       <c r="F938" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G938" t="inlineStr">
@@ -25305,7 +25305,7 @@
       </c>
       <c r="F944" t="inlineStr">
         <is>
-          <t>OH, RP</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G944" t="inlineStr">
@@ -26015,7 +26015,7 @@
       </c>
       <c r="F972" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G972" s="3" t="n">
@@ -26398,7 +26398,7 @@
       </c>
       <c r="F987" t="inlineStr">
         <is>
-          <t>OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G987" s="3" t="n">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="F999" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G999" s="3" t="n">
@@ -26914,7 +26914,7 @@
       </c>
       <c r="F1007" t="inlineStr">
         <is>
-          <t>RE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G1007" s="3" t="n">
@@ -27022,7 +27022,7 @@
       </c>
       <c r="F1011" t="inlineStr">
         <is>
-          <t>NE, SV</t>
+          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
         </is>
       </c>
       <c r="G1011" t="inlineStr">
@@ -27157,7 +27157,7 @@
       </c>
       <c r="F1016" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
         </is>
       </c>
       <c r="G1016" t="inlineStr">
@@ -27317,7 +27317,7 @@
       </c>
       <c r="F1022" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G1022" s="3" t="n">
@@ -27550,7 +27550,7 @@
       </c>
       <c r="F1031" t="inlineStr">
         <is>
-          <t>NE, OH</t>
+          <t>4. Квотация направлена клиенту</t>
         </is>
       </c>
       <c r="G1031" t="inlineStr">

</xml_diff>

<commit_message>
Put the component condition from Cond into the HBS state column.
Quote status still only selects Utair rows. The new state column now lists the offered part conditions, with a price or a price range.

Co-authored-by: alexanderp-cell <alexanderp-cell@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/HBS_List_оборот_с_предложениями.xlsx
+++ b/HBS_List_оборот_с_предложениями.xlsx
@@ -472,7 +472,7 @@
     <col width="11.53125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="7.6640625" bestFit="1" customWidth="1" min="4" max="4"/>
     <col width="26.1328125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="32" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -539,7 +539,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -647,7 +647,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, RP</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1117,7 +1117,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G27" s="3" t="n">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G29" s="3" t="n">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G32" s="3" t="n">
@@ -1476,7 +1476,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>SV, RE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, SV, RP, INSP</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>INSP/TEST</t>
         </is>
       </c>
       <c r="G42" s="3" t="n">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV, RP</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="G50" s="3" t="n">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G51" s="3" t="n">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="G58" s="3" t="n">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес; 7. Клиент согласовал</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>SV, RE</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -2511,7 +2511,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -2831,7 +2831,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес; 7. Клиент согласовал</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3026,7 +3026,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G94" s="3" t="n">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G96" s="3" t="n">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, RP, TEST</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G113" s="3" t="n">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G147" s="3" t="n">
@@ -4728,7 +4728,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, SV, RP, TEST</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G158" s="3" t="n">
@@ -4846,7 +4846,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G161" s="3" t="n">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G164" s="3" t="n">
@@ -4972,7 +4972,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G165" s="3" t="n">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G168" s="3" t="n">
@@ -5238,7 +5238,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G175" s="3" t="n">
@@ -5371,7 +5371,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -5456,7 +5456,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G183" s="3" t="n">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH, RP</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -5759,7 +5759,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G194" s="3" t="n">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G195" s="3" t="n">
@@ -6000,7 +6000,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G203" s="3" t="n">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -6318,7 +6318,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G215" s="3" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="G218" s="3" t="n">
@@ -6434,7 +6434,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G219" s="3" t="n">
@@ -6642,7 +6642,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -6752,7 +6752,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>5. Есть интерес; 7. Клиент согласовал</t>
+          <t>SV, INSP</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -6812,7 +6812,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G233" s="3" t="n">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -7305,7 +7305,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH, SV</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G253" s="3" t="n">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV, RP</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -7658,7 +7658,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G265" s="3" t="n">
@@ -7741,7 +7741,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G270" s="3" t="n">
@@ -7884,7 +7884,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G273" s="3" t="n">
@@ -8092,7 +8092,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G281" s="3" t="n">
@@ -8825,7 +8825,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G310" s="3" t="n">
@@ -9058,7 +9058,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G319" s="3" t="n">
@@ -9091,7 +9091,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G320" s="3" t="n">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G325" s="3" t="n">
@@ -9432,7 +9432,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -9667,7 +9667,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -9727,7 +9727,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G344" s="3" t="n">
@@ -10310,7 +10310,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G367" s="3" t="n">
@@ -10393,7 +10393,7 @@
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV, RP</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -10628,7 +10628,7 @@
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G379" s="3" t="n">
@@ -10686,7 +10686,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, RP</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -10956,7 +10956,7 @@
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -11116,7 +11116,7 @@
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="G401" s="3" t="n">
@@ -11459,7 +11459,7 @@
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G410" s="3" t="n">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -11627,7 +11627,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G416" s="3" t="n">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>NE, OH, SV, RP, INSP, INSP/TEST</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -11745,7 +11745,7 @@
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -11830,7 +11830,7 @@
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -11890,7 +11890,7 @@
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G425" s="3" t="n">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G426" s="3" t="n">
@@ -12206,7 +12206,7 @@
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G437" s="3" t="n">
@@ -12389,7 +12389,7 @@
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G444" s="3" t="n">
@@ -12647,7 +12647,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G454" s="3" t="n">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH, SV</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -13450,7 +13450,7 @@
       </c>
       <c r="F485" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G485" s="3" t="n">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G486" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G488" s="3" t="n">
@@ -14401,7 +14401,7 @@
       </c>
       <c r="F522" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>SV, RP, INSP</t>
         </is>
       </c>
       <c r="G522" t="inlineStr">
@@ -15061,7 +15061,7 @@
       </c>
       <c r="F548" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G548" s="3" t="n">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G551" t="inlineStr">
@@ -15679,7 +15679,7 @@
       </c>
       <c r="F572" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>SV, RP</t>
         </is>
       </c>
       <c r="G572" t="inlineStr">
@@ -16314,7 +16314,7 @@
       </c>
       <c r="F597" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV, INSP, TEST</t>
         </is>
       </c>
       <c r="G597" t="inlineStr">
@@ -16474,7 +16474,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G603" s="3" t="n">
@@ -16557,7 +16557,7 @@
       </c>
       <c r="F606" t="inlineStr">
         <is>
-          <t>5. Есть интерес</t>
+          <t>SV, RP</t>
         </is>
       </c>
       <c r="G606" s="3" t="n">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="F614" t="inlineStr">
         <is>
-          <t>7. Клиент согласовал</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G614" s="3" t="n">
@@ -17423,7 +17423,7 @@
       </c>
       <c r="F640" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G640" s="3" t="n">
@@ -17856,7 +17856,7 @@
       </c>
       <c r="F657" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, SV</t>
         </is>
       </c>
       <c r="G657" t="inlineStr">
@@ -17966,7 +17966,7 @@
       </c>
       <c r="F661" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G661" s="3" t="n">
@@ -18124,7 +18124,7 @@
       </c>
       <c r="F667" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G667" s="3" t="n">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="F672" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G672" t="inlineStr">
@@ -18542,7 +18542,7 @@
       </c>
       <c r="F683" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G683" s="3" t="n">
@@ -18625,7 +18625,7 @@
       </c>
       <c r="F686" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G686" t="inlineStr">
@@ -19285,7 +19285,7 @@
       </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>OH, SV, RP</t>
         </is>
       </c>
       <c r="G712" t="inlineStr">
@@ -19445,7 +19445,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G718" s="3" t="n">
@@ -19528,7 +19528,7 @@
       </c>
       <c r="F721" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G721" s="3" t="n">
@@ -19561,7 +19561,7 @@
       </c>
       <c r="F722" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G722" s="3" t="n">
@@ -19819,7 +19819,7 @@
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G732" t="inlineStr">
@@ -20004,7 +20004,7 @@
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G739" s="3" t="n">
@@ -20212,7 +20212,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RE</t>
         </is>
       </c>
       <c r="G747" t="inlineStr">
@@ -20297,7 +20297,7 @@
       </c>
       <c r="F750" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G750" s="3" t="n">
@@ -20580,7 +20580,7 @@
       </c>
       <c r="F761" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G761" s="3" t="n">
@@ -20763,7 +20763,7 @@
       </c>
       <c r="F768" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G768" s="3" t="n">
@@ -20821,7 +20821,7 @@
       </c>
       <c r="F770" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RE</t>
         </is>
       </c>
       <c r="G770" t="inlineStr">
@@ -21106,7 +21106,7 @@
       </c>
       <c r="F781" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, SV</t>
         </is>
       </c>
       <c r="G781" t="inlineStr">
@@ -21516,7 +21516,7 @@
       </c>
       <c r="F797" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G797" s="3" t="n">
@@ -22249,7 +22249,7 @@
       </c>
       <c r="F826" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G826" s="3" t="n">
@@ -22382,7 +22382,7 @@
       </c>
       <c r="F831" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G831" t="inlineStr">
@@ -22417,7 +22417,7 @@
       </c>
       <c r="F832" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G832" t="inlineStr">
@@ -22852,7 +22852,7 @@
       </c>
       <c r="F849" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G849" s="3" t="n">
@@ -22960,7 +22960,7 @@
       </c>
       <c r="F853" t="inlineStr">
         <is>
-          <t>7. Клиент согласовал</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G853" s="3" t="n">
@@ -23018,7 +23018,7 @@
       </c>
       <c r="F855" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G855" s="3" t="n">
@@ -23051,7 +23051,7 @@
       </c>
       <c r="F856" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G856" s="3" t="n">
@@ -23134,7 +23134,7 @@
       </c>
       <c r="F859" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>OH, SV, TEST</t>
         </is>
       </c>
       <c r="G859" t="inlineStr">
@@ -24619,7 +24619,7 @@
       </c>
       <c r="F918" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RP</t>
         </is>
       </c>
       <c r="G918" s="3" t="n">
@@ -24952,7 +24952,7 @@
       </c>
       <c r="F931" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="G931" s="3" t="n">
@@ -25110,7 +25110,7 @@
       </c>
       <c r="F937" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>FN, OH</t>
         </is>
       </c>
       <c r="G937" t="inlineStr">
@@ -25145,7 +25145,7 @@
       </c>
       <c r="F938" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G938" t="inlineStr">
@@ -25305,7 +25305,7 @@
       </c>
       <c r="F944" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH, RP</t>
         </is>
       </c>
       <c r="G944" t="inlineStr">
@@ -26015,7 +26015,7 @@
       </c>
       <c r="F972" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G972" s="3" t="n">
@@ -26398,7 +26398,7 @@
       </c>
       <c r="F987" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="G987" s="3" t="n">
@@ -26706,7 +26706,7 @@
       </c>
       <c r="F999" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G999" s="3" t="n">
@@ -26914,7 +26914,7 @@
       </c>
       <c r="F1007" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>RE</t>
         </is>
       </c>
       <c r="G1007" s="3" t="n">
@@ -27022,7 +27022,7 @@
       </c>
       <c r="F1011" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 5. Есть интерес</t>
+          <t>NE, SV</t>
         </is>
       </c>
       <c r="G1011" t="inlineStr">
@@ -27157,7 +27157,7 @@
       </c>
       <c r="F1016" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту; 7. Клиент согласовал</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G1016" t="inlineStr">
@@ -27317,7 +27317,7 @@
       </c>
       <c r="F1022" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="G1022" s="3" t="n">
@@ -27550,7 +27550,7 @@
       </c>
       <c r="F1031" t="inlineStr">
         <is>
-          <t>4. Квотация направлена клиенту</t>
+          <t>NE, OH</t>
         </is>
       </c>
       <c r="G1031" t="inlineStr">

</xml_diff>